<commit_message>
added help text for lat and long columns
</commit_message>
<xml_diff>
--- a/app/assets/documents/ingest_manifest_template.xlsx
+++ b/app/assets/documents/ingest_manifest_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10410"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/vagrant/morphosource-vagrant/MorphoSource_SF/app/assets/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{458348A6-0E7E-F64B-BFB9-6E9157EE29B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE0CFD3-4536-0448-882B-43F968FDC12E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="32000" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="246">
   <si>
     <t>Field Section</t>
   </si>
@@ -825,6 +825,9 @@
   <si>
     <t>imaging_event.ct.ie_filter</t>
   </si>
+  <si>
+    <t>Please convert geographic coordinates to decimal if needed</t>
+  </si>
 </sst>
 </file>
 
@@ -959,7 +962,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -1045,6 +1048,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1842,8 +1848,12 @@
       <c r="AH3" s="8"/>
       <c r="AI3" s="8"/>
       <c r="AJ3" s="30"/>
-      <c r="AK3" s="30"/>
-      <c r="AL3" s="30"/>
+      <c r="AK3" s="59" t="s">
+        <v>245</v>
+      </c>
+      <c r="AL3" s="59" t="s">
+        <v>245</v>
+      </c>
       <c r="AM3" s="30"/>
       <c r="AN3" s="30"/>
       <c r="AO3" s="30"/>

</xml_diff>

<commit_message>
create tags param from keyword
</commit_message>
<xml_diff>
--- a/app/assets/documents/ingest_manifest_template.xlsx
+++ b/app/assets/documents/ingest_manifest_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/vagrant/morphosource-vagrant/MorphoSource_SF/app/assets/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE0CFD3-4536-0448-882B-43F968FDC12E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C59A27DB-0F44-6E41-8CDA-794C252B0B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="32000" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="247">
   <si>
     <t>Field Section</t>
   </si>
@@ -828,6 +828,9 @@
   <si>
     <t>Please convert geographic coordinates to decimal if needed</t>
   </si>
+  <si>
+    <t>Value(s) must be letters, accented letters, numbers, and spaces.  Use commas has separators.</t>
+  </si>
 </sst>
 </file>
 
@@ -1823,7 +1826,9 @@
       <c r="U3" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="V3" s="27"/>
+      <c r="V3" s="27" t="s">
+        <v>246</v>
+      </c>
       <c r="W3" s="5"/>
       <c r="X3" s="5"/>
       <c r="Y3" s="29" t="s">

</xml_diff>

<commit_message>
added sample data to batch submission template
</commit_message>
<xml_diff>
--- a/app/assets/documents/ingest_manifest_template.xlsx
+++ b/app/assets/documents/ingest_manifest_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/vagrant/morphosource-vagrant/MorphoSource/app/assets/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5482A66-D75B-274E-B211-D92EAAB303E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF61082C-B38A-D642-81F4-31ACA609FEE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="32000" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="32000" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="266">
   <si>
     <t>Field Section</t>
   </si>
@@ -831,6 +831,63 @@
   <si>
     <t>Media filename or remote file path</t>
   </si>
+  <si>
+    <t>derived</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>raw</t>
+  </si>
+  <si>
+    <t>ABC-123-arm.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTImageSeries </t>
+  </si>
+  <si>
+    <t>Arm</t>
+  </si>
+  <si>
+    <t>Reconstructed image stack</t>
+  </si>
+  <si>
+    <t>male</t>
+  </si>
+  <si>
+    <t>Lemur</t>
+  </si>
+  <si>
+    <t>catta</t>
+  </si>
+  <si>
+    <t>John Smith</t>
+  </si>
+  <si>
+    <t>Avizo</t>
+  </si>
+  <si>
+    <t>Crop</t>
+  </si>
+  <si>
+    <t>ABC-123-arm.stl</t>
+  </si>
+  <si>
+    <t>ABC-123-arm.jpeg</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>Reconstructed tomography to Mesh</t>
+  </si>
+  <si>
+    <t>Left</t>
+  </si>
 </sst>
 </file>
 
@@ -965,7 +1022,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1022,6 +1079,10 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1241,7 +1302,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:CH991"/>
+  <dimension ref="A1:CH989"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="31.1640625" customWidth="1"/>
@@ -2694,20 +2755,31 @@
     <row r="8" spans="1:86" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="27"/>
       <c r="B8" s="26"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="24"/>
-      <c r="G8" s="28"/>
+      <c r="C8" s="24" t="s">
+        <v>251</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>252</v>
+      </c>
+      <c r="F8" s="33" t="s">
+        <v>250</v>
+      </c>
       <c r="H8" s="28"/>
-      <c r="I8" s="24"/>
+      <c r="I8" s="24">
+        <v>203123</v>
+      </c>
       <c r="J8" s="24"/>
       <c r="K8" s="24"/>
       <c r="L8" s="24"/>
       <c r="M8" s="24"/>
       <c r="N8" s="24"/>
-      <c r="O8" s="24"/>
+      <c r="O8" s="24" t="s">
+        <v>253</v>
+      </c>
       <c r="P8" s="24"/>
-      <c r="Q8" s="24"/>
+      <c r="Q8" s="24" t="s">
+        <v>265</v>
+      </c>
       <c r="R8" s="24"/>
       <c r="S8" s="27"/>
       <c r="T8" s="27"/>
@@ -2715,12 +2787,22 @@
       <c r="V8" s="28"/>
       <c r="W8" s="28"/>
       <c r="X8" s="28"/>
-      <c r="Y8" s="27"/>
-      <c r="Z8" s="27"/>
-      <c r="AA8" s="27"/>
+      <c r="Y8" s="27">
+        <v>0.123456</v>
+      </c>
+      <c r="Z8" s="27">
+        <v>0.123456</v>
+      </c>
+      <c r="AA8" s="27">
+        <v>0.123456</v>
+      </c>
       <c r="AB8" s="27"/>
-      <c r="AC8" s="27"/>
-      <c r="AD8" s="24"/>
+      <c r="AC8" s="34" t="s">
+        <v>254</v>
+      </c>
+      <c r="AD8" s="24" t="s">
+        <v>248</v>
+      </c>
       <c r="AE8" s="27"/>
       <c r="AF8" s="24"/>
       <c r="AG8" s="24"/>
@@ -2733,10 +2815,18 @@
       <c r="AN8" s="24"/>
       <c r="AO8" s="24"/>
       <c r="AP8" s="24"/>
-      <c r="AQ8" s="24"/>
-      <c r="AR8" s="24"/>
-      <c r="AS8" s="24"/>
-      <c r="AT8" s="24"/>
+      <c r="AQ8" s="24" t="s">
+        <v>255</v>
+      </c>
+      <c r="AR8" s="24" t="s">
+        <v>249</v>
+      </c>
+      <c r="AS8" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="AT8" s="24" t="s">
+        <v>257</v>
+      </c>
       <c r="AU8" s="24"/>
       <c r="AV8" s="24"/>
       <c r="AW8" s="24"/>
@@ -2745,12 +2835,19 @@
       <c r="AZ8" s="27"/>
       <c r="BA8" s="24"/>
       <c r="BB8" s="24"/>
-      <c r="BC8" s="24"/>
-      <c r="BE8" s="27"/>
+      <c r="BC8" s="24" t="s">
+        <v>249</v>
+      </c>
+      <c r="BE8" s="27">
+        <v>1</v>
+      </c>
       <c r="BF8" s="27"/>
-      <c r="BG8" s="27"/>
-      <c r="BH8" s="27"/>
-      <c r="BI8" s="27"/>
+      <c r="BG8" s="27">
+        <v>100</v>
+      </c>
+      <c r="BI8" s="27">
+        <v>100</v>
+      </c>
       <c r="BJ8" s="24"/>
       <c r="BK8" s="28"/>
       <c r="BL8" s="28"/>
@@ -2772,28 +2869,51 @@
       <c r="CB8" s="28"/>
       <c r="CC8" s="28"/>
       <c r="CD8" s="28"/>
-      <c r="CE8" s="24"/>
+      <c r="CE8" s="24" t="s">
+        <v>258</v>
+      </c>
       <c r="CF8" s="24"/>
-      <c r="CG8" s="24"/>
-      <c r="CH8" s="24"/>
+      <c r="CG8" s="24" t="s">
+        <v>259</v>
+      </c>
+      <c r="CH8" s="24" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="9" spans="1:86" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="27"/>
       <c r="B9" s="26"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="24"/>
-      <c r="G9" s="28"/>
+      <c r="C9" s="24" t="s">
+        <v>261</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>262</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>263</v>
+      </c>
+      <c r="F9" s="33" t="s">
+        <v>247</v>
+      </c>
+      <c r="G9" s="24" t="s">
+        <v>251</v>
+      </c>
       <c r="H9" s="28"/>
-      <c r="I9" s="24"/>
+      <c r="I9" s="24">
+        <v>203123</v>
+      </c>
       <c r="J9" s="24"/>
       <c r="K9" s="24"/>
       <c r="L9" s="24"/>
       <c r="M9" s="24"/>
       <c r="N9" s="24"/>
-      <c r="O9" s="24"/>
+      <c r="O9" s="24" t="s">
+        <v>253</v>
+      </c>
       <c r="P9" s="24"/>
-      <c r="Q9" s="24"/>
+      <c r="Q9" s="24" t="s">
+        <v>265</v>
+      </c>
       <c r="R9" s="24"/>
       <c r="S9" s="27"/>
       <c r="T9" s="27"/>
@@ -2819,10 +2939,18 @@
       <c r="AN9" s="24"/>
       <c r="AO9" s="24"/>
       <c r="AP9" s="24"/>
-      <c r="AQ9" s="24"/>
-      <c r="AR9" s="24"/>
-      <c r="AS9" s="24"/>
-      <c r="AT9" s="24"/>
+      <c r="AQ9" s="24" t="s">
+        <v>255</v>
+      </c>
+      <c r="AR9" s="24" t="s">
+        <v>249</v>
+      </c>
+      <c r="AS9" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="AT9" s="24" t="s">
+        <v>257</v>
+      </c>
       <c r="AU9" s="24"/>
       <c r="AV9" s="24"/>
       <c r="AW9" s="24"/>
@@ -2831,12 +2959,19 @@
       <c r="AZ9" s="27"/>
       <c r="BA9" s="24"/>
       <c r="BB9" s="24"/>
-      <c r="BC9" s="24"/>
-      <c r="BE9" s="27"/>
+      <c r="BC9" s="24" t="s">
+        <v>249</v>
+      </c>
+      <c r="BE9" s="27">
+        <v>1</v>
+      </c>
       <c r="BF9" s="27"/>
-      <c r="BG9" s="27"/>
-      <c r="BH9" s="27"/>
-      <c r="BI9" s="27"/>
+      <c r="BG9" s="27">
+        <v>100</v>
+      </c>
+      <c r="BI9" s="27">
+        <v>100</v>
+      </c>
       <c r="BJ9" s="24"/>
       <c r="BK9" s="28"/>
       <c r="BL9" s="28"/>
@@ -2858,72 +2993,28 @@
       <c r="CB9" s="28"/>
       <c r="CC9" s="28"/>
       <c r="CD9" s="28"/>
-      <c r="CE9" s="24"/>
+      <c r="CE9" s="24" t="s">
+        <v>258</v>
+      </c>
       <c r="CF9" s="24"/>
-      <c r="CG9" s="24"/>
-      <c r="CH9" s="24"/>
-    </row>
-    <row r="10" spans="1:86" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="27"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="24"/>
+      <c r="CG9" s="24" t="s">
+        <v>259</v>
+      </c>
+      <c r="CH9" s="24" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="10" spans="1:86" ht="13" x14ac:dyDescent="0.15">
+      <c r="B10" s="2"/>
+      <c r="C10" s="28"/>
       <c r="D10" s="28"/>
-      <c r="E10" s="24"/>
+      <c r="E10" s="28"/>
       <c r="G10" s="28"/>
       <c r="H10" s="28"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="24"/>
-      <c r="L10" s="24"/>
-      <c r="M10" s="24"/>
-      <c r="N10" s="24"/>
-      <c r="O10" s="24"/>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="24"/>
-      <c r="R10" s="24"/>
-      <c r="S10" s="27"/>
-      <c r="T10" s="27"/>
       <c r="U10" s="28"/>
       <c r="V10" s="28"/>
       <c r="W10" s="28"/>
       <c r="X10" s="28"/>
-      <c r="Y10" s="27"/>
-      <c r="Z10" s="27"/>
-      <c r="AA10" s="27"/>
-      <c r="AB10" s="27"/>
-      <c r="AC10" s="27"/>
-      <c r="AD10" s="24"/>
-      <c r="AE10" s="27"/>
-      <c r="AF10" s="24"/>
-      <c r="AG10" s="24"/>
-      <c r="AH10" s="24"/>
-      <c r="AI10" s="24"/>
-      <c r="AJ10" s="24"/>
-      <c r="AK10" s="24"/>
-      <c r="AL10" s="24"/>
-      <c r="AM10" s="24"/>
-      <c r="AN10" s="24"/>
-      <c r="AO10" s="24"/>
-      <c r="AP10" s="24"/>
-      <c r="AQ10" s="24"/>
-      <c r="AR10" s="24"/>
-      <c r="AS10" s="24"/>
-      <c r="AT10" s="24"/>
-      <c r="AU10" s="24"/>
-      <c r="AV10" s="24"/>
-      <c r="AW10" s="24"/>
-      <c r="AX10" s="27"/>
-      <c r="AY10" s="27"/>
-      <c r="AZ10" s="27"/>
-      <c r="BA10" s="24"/>
-      <c r="BB10" s="24"/>
-      <c r="BC10" s="24"/>
-      <c r="BE10" s="27"/>
-      <c r="BF10" s="27"/>
-      <c r="BG10" s="27"/>
-      <c r="BH10" s="27"/>
-      <c r="BI10" s="27"/>
-      <c r="BJ10" s="24"/>
       <c r="BK10" s="28"/>
       <c r="BL10" s="28"/>
       <c r="BM10" s="28"/>
@@ -2938,16 +3029,9 @@
       <c r="BV10" s="28"/>
       <c r="BW10" s="28"/>
       <c r="BX10" s="28"/>
-      <c r="BY10" s="24"/>
-      <c r="BZ10" s="24"/>
-      <c r="CA10" s="24"/>
       <c r="CB10" s="28"/>
       <c r="CC10" s="28"/>
       <c r="CD10" s="28"/>
-      <c r="CE10" s="24"/>
-      <c r="CF10" s="24"/>
-      <c r="CG10" s="24"/>
-      <c r="CH10" s="24"/>
     </row>
     <row r="11" spans="1:86" ht="13" x14ac:dyDescent="0.15">
       <c r="B11" s="2"/>
@@ -31313,64 +31397,6 @@
     </row>
     <row r="989" spans="2:82" ht="13" x14ac:dyDescent="0.15">
       <c r="B989" s="2"/>
-      <c r="C989" s="28"/>
-      <c r="D989" s="28"/>
-      <c r="E989" s="28"/>
-      <c r="G989" s="28"/>
-      <c r="H989" s="28"/>
-      <c r="U989" s="28"/>
-      <c r="V989" s="28"/>
-      <c r="W989" s="28"/>
-      <c r="X989" s="28"/>
-      <c r="BK989" s="28"/>
-      <c r="BL989" s="28"/>
-      <c r="BM989" s="28"/>
-      <c r="BN989" s="28"/>
-      <c r="BO989" s="28"/>
-      <c r="BP989" s="28"/>
-      <c r="BQ989" s="28"/>
-      <c r="BR989" s="28"/>
-      <c r="BS989" s="28"/>
-      <c r="BT989" s="28"/>
-      <c r="BU989" s="28"/>
-      <c r="BV989" s="28"/>
-      <c r="BW989" s="28"/>
-      <c r="BX989" s="28"/>
-      <c r="CB989" s="28"/>
-      <c r="CC989" s="28"/>
-      <c r="CD989" s="28"/>
-    </row>
-    <row r="990" spans="2:82" ht="13" x14ac:dyDescent="0.15">
-      <c r="B990" s="2"/>
-      <c r="C990" s="28"/>
-      <c r="D990" s="28"/>
-      <c r="E990" s="28"/>
-      <c r="G990" s="28"/>
-      <c r="H990" s="28"/>
-      <c r="U990" s="28"/>
-      <c r="V990" s="28"/>
-      <c r="W990" s="28"/>
-      <c r="X990" s="28"/>
-      <c r="BK990" s="28"/>
-      <c r="BL990" s="28"/>
-      <c r="BM990" s="28"/>
-      <c r="BN990" s="28"/>
-      <c r="BO990" s="28"/>
-      <c r="BP990" s="28"/>
-      <c r="BQ990" s="28"/>
-      <c r="BR990" s="28"/>
-      <c r="BS990" s="28"/>
-      <c r="BT990" s="28"/>
-      <c r="BU990" s="28"/>
-      <c r="BV990" s="28"/>
-      <c r="BW990" s="28"/>
-      <c r="BX990" s="28"/>
-      <c r="CB990" s="28"/>
-      <c r="CC990" s="28"/>
-      <c r="CD990" s="28"/>
-    </row>
-    <row r="991" spans="2:82" ht="13" x14ac:dyDescent="0.15">
-      <c r="B991" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>